<commit_message>
Fixed all the bugs related to auth
</commit_message>
<xml_diff>
--- a/output/announcements_10052026.xlsx
+++ b/output/announcements_10052026.xlsx
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -735,12 +735,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>10-May-2026 12:22:18</t>
+          <t>10-May-2026 20:28:22</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>PAISALO</t>
+          <t>MFSL</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr"/>
@@ -750,13 +750,13 @@
       <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>49.49</t>
+          <t>1695</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Non Banking Financial Company (NBFC)</t>
+          <t>Life Insurance</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr"/>
@@ -768,7 +768,7 @@
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=PAISALO&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/Max_10052026202757_POSTALBALLOTRESULTS10052026.pdf</t>
         </is>
       </c>
     </row>
@@ -778,12 +778,12 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>10-May-2026 12:21:19</t>
+          <t>10-May-2026 19:56:48</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>MODINATUR</t>
+          <t>ADANIGREEN</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr"/>
@@ -793,13 +793,13 @@
       <c r="H4" s="7" t="inlineStr"/>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>370.35</t>
+          <t>1350</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr"/>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>Other Agricultural Products</t>
+          <t>Power Generation</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr"/>
@@ -811,7 +811,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=MODINATUR&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/ADANIGREEN_10052026195613_Letters.pdf</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>10-May-2026 12:20:53</t>
+          <t>10-May-2026 19:56:34</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=PAISALO&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/PAISALO_10052026195626_BSE_NSE_Press_Release_110052026.pdf</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>10-May-2026 12:15:38</t>
+          <t>10-May-2026 19:52:01</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=PAISALO&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/PAISALO_10052026195146_BSE_NSE_Investor_Presentation.pdf</t>
         </is>
       </c>
     </row>
@@ -907,12 +907,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>10-May-2026 12:12:59</t>
+          <t>10-May-2026 19:46:29</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>PAISALO</t>
+          <t>RENUKA</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr"/>
@@ -922,13 +922,13 @@
       <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>49.49</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Non Banking Financial Company (NBFC)</t>
+          <t>Sugar</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr"/>
@@ -940,7 +940,7 @@
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=PAISALO&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/RENUKA_10052026194616_NPM26signed.pdf</t>
         </is>
       </c>
     </row>
@@ -950,12 +950,12 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>10-May-2026 12:05:38</t>
+          <t>10-May-2026 19:12:35</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>CMSINFO</t>
+          <t>ORIENTCEM</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr"/>
@@ -965,13 +965,13 @@
       <c r="H8" s="7" t="inlineStr"/>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>290.5</t>
+          <t>141.08</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Diversified Commercial Services</t>
+          <t>Cement &amp; Cement Products</t>
         </is>
       </c>
       <c r="L8" s="8" t="inlineStr"/>
@@ -983,7 +983,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=CMSINFO&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/ORIENTCEM_10052026191141_OCL_Transcript_10052026.pdf</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>10-May-2026 12:02:46</t>
+          <t>10-May-2026 18:51:46</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>IIFLCAPS</t>
+          <t>PTCIL</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr"/>
@@ -1008,13 +1008,13 @@
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>16770</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Stockbroking &amp; Allied</t>
+          <t>Other Industrial Products</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr"/>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=IIFLCAPS&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/PTCINDUSTRIES_10052026185114_Captial_Group_visit_Intimaton_15052026.pdf</t>
         </is>
       </c>
     </row>
@@ -1036,12 +1036,12 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>10-May-2026 11:56:25</t>
+          <t>10-May-2026 18:43:59</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>HINDCOPPER</t>
+          <t>PYRAMID</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
@@ -1051,13 +1051,13 @@
       <c r="H10" s="7" t="inlineStr"/>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>568.9</t>
+          <t>175.01</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr"/>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="L10" s="8" t="inlineStr"/>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=HINDCOPPER&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/PYRAMIDTECHNO_10052026184105_Investor_meeting_Initimation.pdf</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>10-May-2026 11:45:07</t>
+          <t>10-May-2026 18:24:38</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>LICHSGFIN</t>
+          <t>URBANCO</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr"/>
@@ -1094,13 +1094,13 @@
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>581.85</t>
+          <t>137.8</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Housing Finance Company</t>
+          <t>E-Retail/ E-Commerce</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=LICHSGFIN&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/URBANCO_10052026182357_UC_Transcript_May082026.pdf</t>
         </is>
       </c>
     </row>
@@ -1122,12 +1122,12 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>10-May-2026 11:34:15</t>
+          <t>10-May-2026 18:15:52</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>VASCONEQ</t>
+          <t>EFCIL</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr"/>
@@ -1137,13 +1137,13 @@
       <c r="H12" s="7" t="inlineStr"/>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>39.72</t>
+          <t>188.31</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr"/>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Residential Commercial Projects</t>
+          <t>Diversified Commercial Services</t>
         </is>
       </c>
       <c r="L12" s="8" t="inlineStr"/>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=VASCONEQ&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/EFCILTD_10052026181531_EFC__I__-_Newspaper_Intimation_Right_Issues_-_Final.pdf</t>
         </is>
       </c>
     </row>
@@ -1165,12 +1165,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>10-May-2026 11:14:45</t>
+          <t>10-May-2026 17:47:33</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>HOMEFIRST</t>
+          <t>WINDMACHIN</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
@@ -1180,13 +1180,13 @@
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>1200.6</t>
+          <t>316.4</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Housing Finance Company</t>
+          <t>Industrial Products</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr"/>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=HOMEFIRST&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/WINDMACHIN_ROID_85141_KMP_Doc.zip</t>
         </is>
       </c>
     </row>
@@ -1208,12 +1208,12 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>10-May-2026 11:07:15</t>
+          <t>10-May-2026 17:43:06</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>IFCI</t>
+          <t>MAYURUNIQ</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr"/>
@@ -1223,13 +1223,13 @@
       <c r="H14" s="7" t="inlineStr"/>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>64.39</t>
+          <t>630</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr"/>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>Financial Institution</t>
+          <t>Leather And Leather Products</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=IFCI&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/MAYURUNIQ_10052026174044_Disclosure_for_Strike_sd.pdf</t>
         </is>
       </c>
     </row>
@@ -1251,12 +1251,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>10-May-2026 10:28:07</t>
+          <t>10-May-2026 16:46:40</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>ARTEMISMED</t>
+          <t>GUJGASLTD</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr"/>
@@ -1266,13 +1266,13 @@
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>266</t>
+          <t>396.55</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Hospital</t>
+          <t>LPG/CNG/PNG/LNG Supplier</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr"/>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
-          <t>https://www.nseindia.com/api/corporate-announcements?symbol=ARTEMISMED&amp;an_num=</t>
+          <t>https://nsearchives.nseindia.com/corporate/GUJGASLTD_10052026164557_1565newspaperAdvt10052026.pdf</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>2026-05-10T12:24:43.823</t>
+          <t>10-May-2026 16:29:09</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Modi Naturals Ltd</t>
+          <t>MFSL</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr"/>
@@ -1309,11 +1309,15 @@
       <c r="H16" s="7" t="inlineStr"/>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>376.15</t>
+          <t>1695</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr"/>
-      <c r="K16" s="7" t="inlineStr"/>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>Life Insurance</t>
+        </is>
+      </c>
       <c r="L16" s="8" t="inlineStr"/>
       <c r="M16" s="8" t="inlineStr"/>
       <c r="N16" s="6" t="inlineStr">
@@ -1323,7 +1327,7 @@
       </c>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/f5dc4ada-c1ce-4d8c-a48b-8acf7e51bb8c.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/Max_10052026162813_SEDEARNINGCALLCAN10052026.pdf</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1337,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>2026-05-10T12:16:31.957</t>
+          <t>10-May-2026 16:23:12</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Paisalo Digital Ltd</t>
+          <t>NIACL</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr"/>
@@ -1348,11 +1352,15 @@
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>49.46</t>
+          <t>163.38</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
-      <c r="K17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>General Insurance</t>
+        </is>
+      </c>
       <c r="L17" s="5" t="inlineStr"/>
       <c r="M17" s="5" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr">
@@ -1362,7 +1370,7 @@
       </c>
       <c r="O17" s="5" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/1900624a-454f-4669-8376-88e1d18454dd.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/NIACL_10052026162210_InvestorsMeetCancellation.pdf</t>
         </is>
       </c>
     </row>
@@ -1372,12 +1380,12 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>2026-05-10T12:14:24.997</t>
+          <t>10-May-2026 16:05:17</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Paisalo Digital Ltd</t>
+          <t>RCOM</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr"/>
@@ -1387,11 +1395,15 @@
       <c r="H18" s="7" t="inlineStr"/>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>49.46</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr"/>
-      <c r="K18" s="7" t="inlineStr"/>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>Telecom - Cellular &amp; Fixed line services</t>
+        </is>
+      </c>
       <c r="L18" s="8" t="inlineStr"/>
       <c r="M18" s="8" t="inlineStr"/>
       <c r="N18" s="6" t="inlineStr">
@@ -1401,7 +1413,7 @@
       </c>
       <c r="O18" s="8" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/9d00d436-0bd8-43d5-b6c7-5f3f366b13f3.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/RCOM_10052026160503_DisclosureCBIVisitGraceThomas09052026.pdf</t>
         </is>
       </c>
     </row>
@@ -1411,12 +1423,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>2026-05-10T12:11:55.907</t>
+          <t>10-May-2026 15:42:01</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Paisalo Digital Ltd</t>
+          <t>AMBUJACEM</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr"/>
@@ -1426,11 +1438,15 @@
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>49.46</t>
+          <t>443.9</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Cement &amp; Cement Products</t>
+        </is>
+      </c>
       <c r="L19" s="5" t="inlineStr"/>
       <c r="M19" s="5" t="inlineStr"/>
       <c r="N19" s="6" t="inlineStr">
@@ -1440,7 +1456,7 @@
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/86151cc1-336c-4982-9e41-966f48eb5b74.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/AMBUJACEM_10052026154110_ACL_Transcript_Merged.pdf</t>
         </is>
       </c>
     </row>
@@ -1450,36 +1466,52 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>2026-05-10T12:10:03.6</t>
+          <t>10-May-2026 15:35:39</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Paisalo Digital Ltd</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr"/>
+          <t>PAISALO</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>10-05-2026</t>
+        </is>
+      </c>
       <c r="E20" s="7" t="inlineStr"/>
       <c r="F20" s="7" t="inlineStr"/>
       <c r="G20" s="7" t="inlineStr"/>
       <c r="H20" s="7" t="inlineStr"/>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>49.46</t>
+          <t>49.49</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr"/>
-      <c r="K20" s="7" t="inlineStr"/>
-      <c r="L20" s="8" t="inlineStr"/>
-      <c r="M20" s="8" t="inlineStr"/>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>Non Banking Financial Company (NBFC)</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>Paisalo Digital's audited financial results show a significant increase in interest income</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>The company's financial expenses have increased, which may impact profitability</t>
+        </is>
+      </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="O20" s="8" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/f3a30cd5-5da1-40c8-85bd-37e7c2ffe7fa.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/PAISALO_10052026153142_BSE_NSE_Outcome_Results.pdf</t>
         </is>
       </c>
     </row>
@@ -1489,12 +1521,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>2026-05-10T12:09:44.93</t>
+          <t>10-May-2026 15:32:45</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>IIFL Capital Services Ltd</t>
+          <t>MEDIASSIST</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr"/>
@@ -1504,11 +1536,15 @@
       <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>356.50</t>
+          <t>376</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Insurance Distributors</t>
+        </is>
+      </c>
       <c r="L21" s="5" t="inlineStr"/>
       <c r="M21" s="5" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr">
@@ -1518,7 +1554,7 @@
       </c>
       <c r="O21" s="5" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/af66aba8-05e8-4eb8-9f53-3f9727277d80.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/MEDIASSIST_10052026153059_MAHSNewspaperAdvertisment.pdf</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1564,12 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>2026-05-10T12:03:58.943</t>
+          <t>10-May-2026 15:26:31</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Paisalo Digital Ltd</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr"/>
@@ -1543,11 +1579,15 @@
       <c r="H22" s="7" t="inlineStr"/>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>49.46</t>
+          <t>1393</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr"/>
-      <c r="K22" s="7" t="inlineStr"/>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>Cement &amp; Cement Products</t>
+        </is>
+      </c>
       <c r="L22" s="8" t="inlineStr"/>
       <c r="M22" s="8" t="inlineStr"/>
       <c r="N22" s="6" t="inlineStr">
@@ -1557,7 +1597,7 @@
       </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/bac402f5-318d-4694-9f5c-08cbb1a03e9b.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/ACC_1_10052026152606_ACC_Transcript_Revised_F.pdf</t>
         </is>
       </c>
     </row>
@@ -1567,12 +1607,12 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>2026-05-10T11:59:12.83</t>
+          <t>10-May-2026 15:15:44</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>CMS Info Systems Ltd</t>
+          <t>LTTS</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr"/>
@@ -1582,11 +1622,15 @@
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>290.00</t>
+          <t>3816</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr"/>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>IT Enabled Services</t>
+        </is>
+      </c>
       <c r="L23" s="5" t="inlineStr"/>
       <c r="M23" s="5" t="inlineStr"/>
       <c r="N23" s="6" t="inlineStr">
@@ -1596,7 +1640,7 @@
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/3783798b-cb9e-444a-8988-1148e91390cf.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/LTTS_10052026151503_LTTSPostNewspaperAdv10052026final_sd.pdf</t>
         </is>
       </c>
     </row>
@@ -1606,12 +1650,12 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>2026-05-10T11:53:22.887</t>
+          <t>10-May-2026 15:10:04</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Hindustan Copper Ltd</t>
+          <t>CDSL</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr"/>
@@ -1621,11 +1665,15 @@
       <c r="H24" s="7" t="inlineStr"/>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>569.05</t>
+          <t>1261</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr"/>
-      <c r="K24" s="7" t="inlineStr"/>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>Depositories Clearing Houses and Other Intermediaries</t>
+        </is>
+      </c>
       <c r="L24" s="8" t="inlineStr"/>
       <c r="M24" s="8" t="inlineStr"/>
       <c r="N24" s="6" t="inlineStr">
@@ -1635,7 +1683,7 @@
       </c>
       <c r="O24" s="8" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/69e620c7-326e-4811-a95b-90e4497c2a29.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/CDSL_10052026150325_NSE_Intimation_Allotment_Final.pdf</t>
         </is>
       </c>
     </row>
@@ -1645,12 +1693,12 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>2026-05-10T11:51:04.577</t>
+          <t>10-May-2026 15:09:54</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>LIC Housing Finance Ltd</t>
+          <t>DBOL</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
@@ -1660,11 +1708,15 @@
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>581.30</t>
+          <t>119</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr"/>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Sugar</t>
+        </is>
+      </c>
       <c r="L25" s="5" t="inlineStr"/>
       <c r="M25" s="5" t="inlineStr"/>
       <c r="N25" s="6" t="inlineStr">
@@ -1674,7 +1726,7 @@
       </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/46c37883-7f04-4d8b-b386-949663263fc9.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/DBOLTD_10052026150943_Intimation_ED.pdf</t>
         </is>
       </c>
     </row>
@@ -1684,12 +1736,12 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>2026-05-10T11:38:21.34</t>
+          <t>10-May-2026 14:43:13</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Vascon Engineers Ltd</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr"/>
@@ -1699,11 +1751,15 @@
       <c r="H26" s="7" t="inlineStr"/>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>39.94</t>
+          <t>130</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr"/>
-      <c r="K26" s="7" t="inlineStr"/>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>Iron &amp; Steel Products</t>
+        </is>
+      </c>
       <c r="L26" s="8" t="inlineStr"/>
       <c r="M26" s="8" t="inlineStr"/>
       <c r="N26" s="6" t="inlineStr">
@@ -1713,7 +1769,7 @@
       </c>
       <c r="O26" s="8" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/4fc9fecc-4837-4955-a615-51f5d213b63f.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/SAMBHAV2024_10052026144234_Sambhv_Q4FY26.pdf</t>
         </is>
       </c>
     </row>
@@ -1723,12 +1779,12 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>2026-05-10T11:16:03.83</t>
+          <t>10-May-2026 14:42:54</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>IFCI Ltd</t>
+          <t>NELCAST</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr"/>
@@ -1738,11 +1794,15 @@
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>64.44</t>
+          <t>161.8</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr"/>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>Castings &amp; Forgings</t>
+        </is>
+      </c>
       <c r="L27" s="5" t="inlineStr"/>
       <c r="M27" s="5" t="inlineStr"/>
       <c r="N27" s="6" t="inlineStr">
@@ -1752,7 +1812,7 @@
       </c>
       <c r="O27" s="5" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/6232a51c-63ad-41f3-80a8-6fe4e4d8b855.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/NELCAST1_10052026144212_10052026_newsad_IEPF_signed.pdf</t>
         </is>
       </c>
     </row>
@@ -1762,12 +1822,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>2026-05-10T11:11:24.69</t>
+          <t>10-May-2026 14:34:10</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Home First Finance Company India Ltd</t>
+          <t>MUTHOOTCAP</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr"/>
@@ -1777,11 +1837,15 @@
       <c r="H28" s="7" t="inlineStr"/>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>1200.00</t>
+          <t>223.36</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr"/>
-      <c r="K28" s="7" t="inlineStr"/>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>Non Banking Financial Company (NBFC)</t>
+        </is>
+      </c>
       <c r="L28" s="8" t="inlineStr"/>
       <c r="M28" s="8" t="inlineStr"/>
       <c r="N28" s="6" t="inlineStr">
@@ -1791,7 +1855,7 @@
       </c>
       <c r="O28" s="8" t="inlineStr">
         <is>
-          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/69567c89-3db1-421b-acc0-16c21cf93ed7.pdf</t>
+          <t>https://nsearchives.nseindia.com/corporate/MUTHOOTCAPS_10052026143356_Final.pdf</t>
         </is>
       </c>
     </row>
@@ -1801,12 +1865,12 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>2026-05-10T10:19:58.443</t>
+          <t>10-May-2026 13:12:57</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Artemis Medicare Services Ltd</t>
+          <t>BAJAJHCARE</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr"/>
@@ -1816,11 +1880,15 @@
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>265.35</t>
+          <t>338.45</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr"/>
-      <c r="K29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
       <c r="L29" s="5" t="inlineStr"/>
       <c r="M29" s="5" t="inlineStr"/>
       <c r="N29" s="6" t="inlineStr">
@@ -1829,6 +1897,3237 @@
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/BAJAJHCARE_10052026131122_Intimation_for_Newspaper_Publication_Final.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="55" customHeight="1">
+      <c r="A30" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>10-May-2026 13:05:00</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>PAISALO</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr"/>
+      <c r="E30" s="7" t="inlineStr"/>
+      <c r="F30" s="7" t="inlineStr"/>
+      <c r="G30" s="7" t="inlineStr"/>
+      <c r="H30" s="7" t="inlineStr"/>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>49.49</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="inlineStr"/>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>Non Banking Financial Company (NBFC)</t>
+        </is>
+      </c>
+      <c r="L30" s="8" t="inlineStr"/>
+      <c r="M30" s="8" t="inlineStr"/>
+      <c r="N30" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O30" s="8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/PAISALO_10052026130453_BSE_NSE_Fund_Utilisation.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="55" customHeight="1">
+      <c r="A31" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>10-May-2026 13:00:10</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>FEDERALBNK</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>297.4</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>Private Sector Bank</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr"/>
+      <c r="M31" s="5" t="inlineStr"/>
+      <c r="N31" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O31" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/FEDERALBNK_10052026125954_ESOS_227227_090526_SE_S.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="55" customHeight="1">
+      <c r="A32" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:56:37</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>IFGLEXPOR</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr"/>
+      <c r="E32" s="7" t="inlineStr"/>
+      <c r="F32" s="7" t="inlineStr"/>
+      <c r="G32" s="7" t="inlineStr"/>
+      <c r="H32" s="7" t="inlineStr"/>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>187.38</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr"/>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>Electrodes &amp; Refractories</t>
+        </is>
+      </c>
+      <c r="L32" s="8" t="inlineStr"/>
+      <c r="M32" s="8" t="inlineStr"/>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O32" s="8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/IFGLEXPOR_ROID_85134_KMP_Doc.zip</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="55" customHeight="1">
+      <c r="A33" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:49:18</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>IFGLEXPOR</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>187.38</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>Electrodes &amp; Refractories</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr"/>
+      <c r="M33" s="5" t="inlineStr"/>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/IFGLEXPOR_10052026124839_Disclosure_signed.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="55" customHeight="1">
+      <c r="A34" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:45:07</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>IFGLEXPOR</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr"/>
+      <c r="E34" s="7" t="inlineStr"/>
+      <c r="F34" s="7" t="inlineStr"/>
+      <c r="G34" s="7" t="inlineStr"/>
+      <c r="H34" s="7" t="inlineStr"/>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>187.38</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr"/>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>Electrodes &amp; Refractories</t>
+        </is>
+      </c>
+      <c r="L34" s="8" t="inlineStr"/>
+      <c r="M34" s="8" t="inlineStr"/>
+      <c r="N34" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O34" s="8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/IFGLEXPOR_10052026124417_Disclosure_signed.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="55" customHeight="1">
+      <c r="A35" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:22:18</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>PAISALO</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>49.49</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>Non Banking Financial Company (NBFC)</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr"/>
+      <c r="M35" s="5" t="inlineStr"/>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O35" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/PAISALO_10052026122211_BSE_NSE_Outcome_10052026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="55" customHeight="1">
+      <c r="A36" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:21:19</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>MODINATUR</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr"/>
+      <c r="E36" s="7" t="inlineStr"/>
+      <c r="F36" s="7" t="inlineStr"/>
+      <c r="G36" s="7" t="inlineStr"/>
+      <c r="H36" s="7" t="inlineStr"/>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>370.35</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr"/>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>Other Agricultural Products</t>
+        </is>
+      </c>
+      <c r="L36" s="8" t="inlineStr"/>
+      <c r="M36" s="8" t="inlineStr"/>
+      <c r="N36" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O36" s="8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/MODINATURALS_10052026122045_Final_Intimation.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="55" customHeight="1">
+      <c r="A37" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:20:53</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>PAISALO</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>49.49</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>Non Banking Financial Company (NBFC)</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr"/>
+      <c r="M37" s="5" t="inlineStr"/>
+      <c r="N37" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O37" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/PAISALO_10052026122023_BSE_NSE_Outcome_10052026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="55" customHeight="1">
+      <c r="A38" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:15:38</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>PAISALO</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr"/>
+      <c r="E38" s="7" t="inlineStr"/>
+      <c r="F38" s="7" t="inlineStr"/>
+      <c r="G38" s="7" t="inlineStr"/>
+      <c r="H38" s="7" t="inlineStr"/>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>49.49</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="inlineStr"/>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>Non Banking Financial Company (NBFC)</t>
+        </is>
+      </c>
+      <c r="L38" s="8" t="inlineStr"/>
+      <c r="M38" s="8" t="inlineStr"/>
+      <c r="N38" s="6" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="O38" s="8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/PAISALO_10052026121445_BSE_NSE_Outcome_10052026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="55" customHeight="1">
+      <c r="A39" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:12:59</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>PAISALO</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>49.49</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>Non Banking Financial Company (NBFC)</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr"/>
+      <c r="M39" s="5" t="inlineStr"/>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="O39" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/PAISALO_10052026121058_BSE_NSE_Outcome_Results.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="55" customHeight="1">
+      <c r="A40" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:05:38</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>CMSINFO</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr"/>
+      <c r="E40" s="7" t="inlineStr"/>
+      <c r="F40" s="7" t="inlineStr"/>
+      <c r="G40" s="7" t="inlineStr"/>
+      <c r="H40" s="7" t="inlineStr"/>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>290.5</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="inlineStr"/>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>Diversified Commercial Services</t>
+        </is>
+      </c>
+      <c r="L40" s="8" t="inlineStr"/>
+      <c r="M40" s="8" t="inlineStr"/>
+      <c r="N40" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O40" s="8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/CMSINFO_10052026120508_PressReleaseMay2026sd.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="55" customHeight="1">
+      <c r="A41" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>10-May-2026 12:02:46</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>IIFLCAPS</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>356</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>Stockbroking &amp; Allied</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr"/>
+      <c r="M41" s="5" t="inlineStr"/>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O41" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/IIFLSEC_10052026115938_SEIntimationsigned.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="55" customHeight="1">
+      <c r="A42" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>10-May-2026 11:56:25</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>HINDCOPPER</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr"/>
+      <c r="E42" s="7" t="inlineStr"/>
+      <c r="F42" s="7" t="inlineStr"/>
+      <c r="G42" s="7" t="inlineStr"/>
+      <c r="H42" s="7" t="inlineStr"/>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>568.9</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr"/>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>Copper</t>
+        </is>
+      </c>
+      <c r="L42" s="8" t="inlineStr"/>
+      <c r="M42" s="8" t="inlineStr"/>
+      <c r="N42" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O42" s="8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/HINDCOPPERMKD_10052026115605_Reg30_AppointmentofShriGDGupta.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="55" customHeight="1">
+      <c r="A43" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>10-May-2026 11:45:07</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>LICHSGFIN</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>581.85</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>Housing Finance Company</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr"/>
+      <c r="M43" s="5" t="inlineStr"/>
+      <c r="N43" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O43" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/LICHSGFIN_10052026114444_Change_in_SMP_COO_-_demise.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="55" customHeight="1">
+      <c r="A44" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>10-May-2026 11:34:15</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>VASCONEQ</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr"/>
+      <c r="E44" s="7" t="inlineStr"/>
+      <c r="F44" s="7" t="inlineStr"/>
+      <c r="G44" s="7" t="inlineStr"/>
+      <c r="H44" s="7" t="inlineStr"/>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>39.72</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="inlineStr"/>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>Residential Commercial Projects</t>
+        </is>
+      </c>
+      <c r="L44" s="8" t="inlineStr"/>
+      <c r="M44" s="8" t="inlineStr"/>
+      <c r="N44" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O44" s="8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/VASCONEQ_10052026113346_Cutoffdateintimation_Sd.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="55" customHeight="1">
+      <c r="A45" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>10-May-2026 11:14:45</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>HOMEFIRST</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>1200.6</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>Housing Finance Company</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr"/>
+      <c r="M45" s="5" t="inlineStr"/>
+      <c r="N45" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O45" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/HOMEFIRST_10052026111417_InvestorMeetIntimation10052026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="55" customHeight="1">
+      <c r="A46" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>10-May-2026 11:07:15</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>IFCI</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr"/>
+      <c r="E46" s="7" t="inlineStr"/>
+      <c r="F46" s="7" t="inlineStr"/>
+      <c r="G46" s="7" t="inlineStr"/>
+      <c r="H46" s="7" t="inlineStr"/>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t>64.39</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="inlineStr"/>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>Financial Institution</t>
+        </is>
+      </c>
+      <c r="L46" s="8" t="inlineStr"/>
+      <c r="M46" s="8" t="inlineStr"/>
+      <c r="N46" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O46" s="8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/IFCI_10052026110512_STX_CESSATION_ID_signed.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="55" customHeight="1">
+      <c r="A47" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>10-May-2026 10:28:07</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>ARTEMISMED</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>266</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr"/>
+      <c r="M47" s="5" t="inlineStr"/>
+      <c r="N47" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O47" s="5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/corporate/ARTEMISMED_10052026102350_Disclosure_10_May_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="55" customHeight="1">
+      <c r="A48" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T21:47:36.063</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Zaggle Prepaid Ocean Services Ltd</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr"/>
+      <c r="E48" s="7" t="inlineStr"/>
+      <c r="F48" s="7" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr"/>
+      <c r="H48" s="7" t="inlineStr"/>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>257.65</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr"/>
+      <c r="K48" s="7" t="inlineStr"/>
+      <c r="L48" s="8" t="inlineStr"/>
+      <c r="M48" s="8" t="inlineStr"/>
+      <c r="N48" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O48" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/06bae64d-8807-4688-a8dc-f7be7c4555ee.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="55" customHeight="1">
+      <c r="A49" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T21:17:45.483</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Samtel India Ltd-$</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr"/>
+      <c r="H49" s="4" t="inlineStr"/>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>33.90</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="5" t="inlineStr"/>
+      <c r="M49" s="5" t="inlineStr"/>
+      <c r="N49" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O49" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/8603708f-c5af-4704-894b-7a00bb6fe4f3.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="55" customHeight="1">
+      <c r="A50" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T20:48:01.487</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Deccan Gold Mines Ltd</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr"/>
+      <c r="E50" s="7" t="inlineStr"/>
+      <c r="F50" s="7" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr"/>
+      <c r="H50" s="7" t="inlineStr"/>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>120.95</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr"/>
+      <c r="K50" s="7" t="inlineStr"/>
+      <c r="L50" s="8" t="inlineStr"/>
+      <c r="M50" s="8" t="inlineStr"/>
+      <c r="N50" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O50" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/dc96b420-5e5b-49ca-bf5e-94e978888c51.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="55" customHeight="1">
+      <c r="A51" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T20:46:14.083</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Hampton Sky Realty Ltd</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr"/>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr"/>
+      <c r="H51" s="4" t="inlineStr"/>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>11.50</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr"/>
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="5" t="inlineStr"/>
+      <c r="M51" s="5" t="inlineStr"/>
+      <c r="N51" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O51" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/a3e534d4-bc33-45a5-b4d2-a3fb43d101bf.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="55" customHeight="1">
+      <c r="A52" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T20:18:39.323</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>Max Financial Services Ltd</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr"/>
+      <c r="E52" s="7" t="inlineStr"/>
+      <c r="F52" s="7" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr"/>
+      <c r="H52" s="7" t="inlineStr"/>
+      <c r="I52" s="7" t="inlineStr">
+        <is>
+          <t>1698.40</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr"/>
+      <c r="K52" s="7" t="inlineStr"/>
+      <c r="L52" s="8" t="inlineStr"/>
+      <c r="M52" s="8" t="inlineStr"/>
+      <c r="N52" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O52" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/374ac4a4-26bd-48e5-8a6a-76574f3efae8.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="55" customHeight="1">
+      <c r="A53" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T20:15:01.283</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Jupiter Infomedia Ltd</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr"/>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr"/>
+      <c r="H53" s="4" t="inlineStr"/>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>64.94</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr"/>
+      <c r="K53" s="4" t="inlineStr"/>
+      <c r="L53" s="5" t="inlineStr"/>
+      <c r="M53" s="5" t="inlineStr"/>
+      <c r="N53" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O53" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/d2476742-ac57-4730-83fa-ef0de26c22be.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="55" customHeight="1">
+      <c r="A54" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T19:58:26.98</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Apollo Finvest India Ltd</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr"/>
+      <c r="E54" s="7" t="inlineStr"/>
+      <c r="F54" s="7" t="inlineStr"/>
+      <c r="G54" s="7" t="inlineStr"/>
+      <c r="H54" s="7" t="inlineStr"/>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>369.80</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="inlineStr"/>
+      <c r="K54" s="7" t="inlineStr"/>
+      <c r="L54" s="8" t="inlineStr"/>
+      <c r="M54" s="8" t="inlineStr"/>
+      <c r="N54" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O54" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/96ff099b-3606-47c6-bc0b-edd231e3cc59.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="55" customHeight="1">
+      <c r="A55" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T19:57:00.087</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Adani Green Energy Ltd</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr"/>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr"/>
+      <c r="H55" s="4" t="inlineStr"/>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>1355.80</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr"/>
+      <c r="K55" s="4" t="inlineStr"/>
+      <c r="L55" s="5" t="inlineStr"/>
+      <c r="M55" s="5" t="inlineStr"/>
+      <c r="N55" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O55" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/e60eaf4e-fd82-47ea-83b2-afc08631b3e1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="55" customHeight="1">
+      <c r="A56" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T19:55:03.29</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Ltd</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr"/>
+      <c r="E56" s="7" t="inlineStr"/>
+      <c r="F56" s="7" t="inlineStr"/>
+      <c r="G56" s="7" t="inlineStr"/>
+      <c r="H56" s="7" t="inlineStr"/>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>49.46</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="inlineStr"/>
+      <c r="K56" s="7" t="inlineStr"/>
+      <c r="L56" s="8" t="inlineStr"/>
+      <c r="M56" s="8" t="inlineStr"/>
+      <c r="N56" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O56" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/02d448b7-df5e-4dd6-95e2-c3b5929be6fc.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="55" customHeight="1">
+      <c r="A57" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T19:50:30.81</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Ltd</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr"/>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr"/>
+      <c r="G57" s="4" t="inlineStr"/>
+      <c r="H57" s="4" t="inlineStr"/>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>49.46</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr"/>
+      <c r="K57" s="4" t="inlineStr"/>
+      <c r="L57" s="5" t="inlineStr"/>
+      <c r="M57" s="5" t="inlineStr"/>
+      <c r="N57" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O57" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/7dd14016-f623-445c-b0cd-e1ff1a573157.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="55" customHeight="1">
+      <c r="A58" s="7" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T19:41:10.703</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Shree Renuka Sugars Ltd</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr"/>
+      <c r="E58" s="7" t="inlineStr"/>
+      <c r="F58" s="7" t="inlineStr"/>
+      <c r="G58" s="7" t="inlineStr"/>
+      <c r="H58" s="7" t="inlineStr"/>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>27.60</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr"/>
+      <c r="K58" s="7" t="inlineStr"/>
+      <c r="L58" s="8" t="inlineStr"/>
+      <c r="M58" s="8" t="inlineStr"/>
+      <c r="N58" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O58" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/522ddf2d-1b9d-4dfc-9e54-7f149656cb35.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="55" customHeight="1">
+      <c r="A59" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T19:22:57.01</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Bharti Hexacom Ltd</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr"/>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr"/>
+      <c r="H59" s="4" t="inlineStr"/>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>1498.20</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr"/>
+      <c r="K59" s="4" t="inlineStr"/>
+      <c r="L59" s="5" t="inlineStr"/>
+      <c r="M59" s="5" t="inlineStr"/>
+      <c r="N59" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O59" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/f4da6046-bd55-484e-a36c-8c58ea5296a6.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="55" customHeight="1">
+      <c r="A60" s="7" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T19:20:43.207</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Orient Cement Ltd</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr"/>
+      <c r="E60" s="7" t="inlineStr"/>
+      <c r="F60" s="7" t="inlineStr"/>
+      <c r="G60" s="7" t="inlineStr"/>
+      <c r="H60" s="7" t="inlineStr"/>
+      <c r="I60" s="7" t="inlineStr">
+        <is>
+          <t>141.95</t>
+        </is>
+      </c>
+      <c r="J60" s="7" t="inlineStr"/>
+      <c r="K60" s="7" t="inlineStr"/>
+      <c r="L60" s="8" t="inlineStr"/>
+      <c r="M60" s="8" t="inlineStr"/>
+      <c r="N60" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O60" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/436b5f9d-ef9a-4859-8d5d-10ed20708803.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="55" customHeight="1">
+      <c r="A61" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T19:19:21.163</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Ltd</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr"/>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr"/>
+      <c r="H61" s="4" t="inlineStr"/>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>1834.90</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr"/>
+      <c r="K61" s="4" t="inlineStr"/>
+      <c r="L61" s="5" t="inlineStr"/>
+      <c r="M61" s="5" t="inlineStr"/>
+      <c r="N61" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O61" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/670321a5-5826-40e1-bc69-c3e3674f695e.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="55" customHeight="1">
+      <c r="A62" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T18:56:42.05</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>Dynavision Ltd</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr"/>
+      <c r="E62" s="7" t="inlineStr"/>
+      <c r="F62" s="7" t="inlineStr"/>
+      <c r="G62" s="7" t="inlineStr"/>
+      <c r="H62" s="7" t="inlineStr"/>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>177.00</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr"/>
+      <c r="K62" s="7" t="inlineStr"/>
+      <c r="L62" s="8" t="inlineStr"/>
+      <c r="M62" s="8" t="inlineStr"/>
+      <c r="N62" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O62" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/fc7028b4-fdf6-4da9-a307-0df74ce2eb5a.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="55" customHeight="1">
+      <c r="A63" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T18:54:04.293</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>PTC Industries Ltd</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr"/>
+      <c r="E63" s="4" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr"/>
+      <c r="G63" s="4" t="inlineStr"/>
+      <c r="H63" s="4" t="inlineStr"/>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>16790.45</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr"/>
+      <c r="K63" s="4" t="inlineStr"/>
+      <c r="L63" s="5" t="inlineStr"/>
+      <c r="M63" s="5" t="inlineStr"/>
+      <c r="N63" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O63" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/6e6e1301-783b-4c50-84ef-8f9696596eb2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="55" customHeight="1">
+      <c r="A64" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T18:38:52.3</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>Integrated Capital Services Ltd</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr"/>
+      <c r="E64" s="7" t="inlineStr"/>
+      <c r="F64" s="7" t="inlineStr"/>
+      <c r="G64" s="7" t="inlineStr"/>
+      <c r="H64" s="7" t="inlineStr"/>
+      <c r="I64" s="7" t="inlineStr">
+        <is>
+          <t>5.10</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr"/>
+      <c r="K64" s="7" t="inlineStr"/>
+      <c r="L64" s="8" t="inlineStr"/>
+      <c r="M64" s="8" t="inlineStr"/>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O64" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/3020762f-9173-404e-a57a-263f67110a79.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="55" customHeight="1">
+      <c r="A65" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T18:36:52.777</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Pyramid Technoplast Ltd</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr"/>
+      <c r="E65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr"/>
+      <c r="G65" s="4" t="inlineStr"/>
+      <c r="H65" s="4" t="inlineStr"/>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>176.80</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr"/>
+      <c r="K65" s="4" t="inlineStr"/>
+      <c r="L65" s="5" t="inlineStr"/>
+      <c r="M65" s="5" t="inlineStr"/>
+      <c r="N65" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O65" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/f6964529-790e-4f0d-bd77-5f819d2c6faa.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="55" customHeight="1">
+      <c r="A66" s="7" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T18:30:47.41</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>ASM Technologies Ltd</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr"/>
+      <c r="E66" s="7" t="inlineStr"/>
+      <c r="F66" s="7" t="inlineStr"/>
+      <c r="G66" s="7" t="inlineStr"/>
+      <c r="H66" s="7" t="inlineStr"/>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t>3524.25</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="inlineStr"/>
+      <c r="K66" s="7" t="inlineStr"/>
+      <c r="L66" s="8" t="inlineStr"/>
+      <c r="M66" s="8" t="inlineStr"/>
+      <c r="N66" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O66" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/58e7ab7a-39a7-4bd8-aca9-b42048f94686.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="55" customHeight="1">
+      <c r="A67" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T18:28:53.68</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Urban Company Ltd</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr"/>
+      <c r="E67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr"/>
+      <c r="H67" s="4" t="inlineStr"/>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>139.55</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="5" t="inlineStr"/>
+      <c r="M67" s="5" t="inlineStr"/>
+      <c r="N67" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O67" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/9467ec01-6ac1-4f1d-aa88-552b073557b1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="55" customHeight="1">
+      <c r="A68" s="7" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T18:13:41.67</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>EFC (I) Ltd</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr"/>
+      <c r="E68" s="7" t="inlineStr"/>
+      <c r="F68" s="7" t="inlineStr"/>
+      <c r="G68" s="7" t="inlineStr"/>
+      <c r="H68" s="7" t="inlineStr"/>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>189.65</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="inlineStr"/>
+      <c r="K68" s="7" t="inlineStr"/>
+      <c r="L68" s="8" t="inlineStr"/>
+      <c r="M68" s="8" t="inlineStr"/>
+      <c r="N68" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O68" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/e156996e-6e01-4395-a25c-bb526a0858ab.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="55" customHeight="1">
+      <c r="A69" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T17:39:16.303</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Concord Control Systems Ltd</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr"/>
+      <c r="E69" s="4" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr"/>
+      <c r="G69" s="4" t="inlineStr"/>
+      <c r="H69" s="4" t="inlineStr"/>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>2680.20</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" s="4" t="inlineStr"/>
+      <c r="L69" s="5" t="inlineStr"/>
+      <c r="M69" s="5" t="inlineStr"/>
+      <c r="N69" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O69" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/5286c40c-993a-4661-8545-b7ce9f2f8b7a.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="55" customHeight="1">
+      <c r="A70" s="7" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T17:26:33.58</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>Mayur Uniquoters Ltd-$</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr"/>
+      <c r="E70" s="7" t="inlineStr"/>
+      <c r="F70" s="7" t="inlineStr"/>
+      <c r="G70" s="7" t="inlineStr"/>
+      <c r="H70" s="7" t="inlineStr"/>
+      <c r="I70" s="7" t="inlineStr">
+        <is>
+          <t>629.70</t>
+        </is>
+      </c>
+      <c r="J70" s="7" t="inlineStr"/>
+      <c r="K70" s="7" t="inlineStr"/>
+      <c r="L70" s="8" t="inlineStr"/>
+      <c r="M70" s="8" t="inlineStr"/>
+      <c r="N70" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O70" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/fb45b883-daf1-4b03-a59d-a292ac0d0ed4.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="55" customHeight="1">
+      <c r="A71" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T17:20:37.627</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>DMR Engineering Ltd</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr"/>
+      <c r="E71" s="4" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr"/>
+      <c r="G71" s="4" t="inlineStr"/>
+      <c r="H71" s="4" t="inlineStr"/>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>44.73</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr"/>
+      <c r="K71" s="4" t="inlineStr"/>
+      <c r="L71" s="5" t="inlineStr"/>
+      <c r="M71" s="5" t="inlineStr"/>
+      <c r="N71" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O71" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/8634ac32-1bd5-4650-9e20-eb8d141c5cb7.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="55" customHeight="1">
+      <c r="A72" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T17:00:09.4</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>Credent Global Finance Ltd</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr"/>
+      <c r="E72" s="7" t="inlineStr"/>
+      <c r="F72" s="7" t="inlineStr"/>
+      <c r="G72" s="7" t="inlineStr"/>
+      <c r="H72" s="7" t="inlineStr"/>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>29.14</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr"/>
+      <c r="K72" s="7" t="inlineStr"/>
+      <c r="L72" s="8" t="inlineStr"/>
+      <c r="M72" s="8" t="inlineStr"/>
+      <c r="N72" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O72" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/a853f7b4-deca-41e1-8345-ffe01fa88ea6.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="55" customHeight="1">
+      <c r="A73" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T16:43:29.587</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Gujarat Gas Ltd</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr"/>
+      <c r="E73" s="4" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr"/>
+      <c r="G73" s="4" t="inlineStr"/>
+      <c r="H73" s="4" t="inlineStr"/>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>396.55</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr"/>
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="5" t="inlineStr"/>
+      <c r="M73" s="5" t="inlineStr"/>
+      <c r="N73" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O73" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/2bf9f4b7-7005-4a81-81f2-f22ebc2ad7f2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="55" customHeight="1">
+      <c r="A74" s="7" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T16:39:41.323</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>Popular Estate Management Ltd</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr"/>
+      <c r="E74" s="7" t="inlineStr"/>
+      <c r="F74" s="7" t="inlineStr"/>
+      <c r="G74" s="7" t="inlineStr"/>
+      <c r="H74" s="7" t="inlineStr"/>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>17.00</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr"/>
+      <c r="K74" s="7" t="inlineStr"/>
+      <c r="L74" s="8" t="inlineStr"/>
+      <c r="M74" s="8" t="inlineStr"/>
+      <c r="N74" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O74" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/2ca3f7f3-d751-48bb-8ffd-1d1264d4e398.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="55" customHeight="1">
+      <c r="A75" s="4" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T16:26:15.763</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Max Financial Services Ltd</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr"/>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr"/>
+      <c r="H75" s="4" t="inlineStr"/>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>1698.40</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr"/>
+      <c r="K75" s="4" t="inlineStr"/>
+      <c r="L75" s="5" t="inlineStr"/>
+      <c r="M75" s="5" t="inlineStr"/>
+      <c r="N75" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O75" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/1c968c7a-0d77-4a81-90fd-8d8a1edfed75.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="55" customHeight="1">
+      <c r="A76" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T16:25:42.163</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>The New India Assurance Company Ltd</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr"/>
+      <c r="E76" s="7" t="inlineStr"/>
+      <c r="F76" s="7" t="inlineStr"/>
+      <c r="G76" s="7" t="inlineStr"/>
+      <c r="H76" s="7" t="inlineStr"/>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>164.05</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr"/>
+      <c r="K76" s="7" t="inlineStr"/>
+      <c r="L76" s="8" t="inlineStr"/>
+      <c r="M76" s="8" t="inlineStr"/>
+      <c r="N76" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O76" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/63c12966-0fe2-431f-a3cc-bd21ec29ee39.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="55" customHeight="1">
+      <c r="A77" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T16:14:15.047</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Reliance Communications Ltd</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr"/>
+      <c r="E77" s="4" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr"/>
+      <c r="G77" s="4" t="inlineStr"/>
+      <c r="H77" s="4" t="inlineStr"/>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr"/>
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="5" t="inlineStr"/>
+      <c r="M77" s="5" t="inlineStr"/>
+      <c r="N77" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O77" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/62799944-6a0c-4732-b4e5-14f20a6370c9.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="55" customHeight="1">
+      <c r="A78" s="7" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T16:03:07.377</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>Stallion India Fluorochemicals Ltd</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr"/>
+      <c r="E78" s="7" t="inlineStr"/>
+      <c r="F78" s="7" t="inlineStr"/>
+      <c r="G78" s="7" t="inlineStr"/>
+      <c r="H78" s="7" t="inlineStr"/>
+      <c r="I78" s="7" t="inlineStr">
+        <is>
+          <t>160.85</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="inlineStr"/>
+      <c r="K78" s="7" t="inlineStr"/>
+      <c r="L78" s="8" t="inlineStr"/>
+      <c r="M78" s="8" t="inlineStr"/>
+      <c r="N78" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O78" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/957552e7-68c5-4761-b398-8a9179c7caff.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="55" customHeight="1">
+      <c r="A79" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:59:41.157</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Hypersoft Technologies Ltd</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr"/>
+      <c r="E79" s="4" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr"/>
+      <c r="H79" s="4" t="inlineStr"/>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>134.75</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr"/>
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="5" t="inlineStr"/>
+      <c r="M79" s="5" t="inlineStr"/>
+      <c r="N79" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O79" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/dfb62ead-14a1-4092-8da6-0e368e0ec358.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="55" customHeight="1">
+      <c r="A80" s="7" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:36:19.44</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>Medi Assist Healthcare Services Ltd</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr"/>
+      <c r="E80" s="7" t="inlineStr"/>
+      <c r="F80" s="7" t="inlineStr"/>
+      <c r="G80" s="7" t="inlineStr"/>
+      <c r="H80" s="7" t="inlineStr"/>
+      <c r="I80" s="7" t="inlineStr">
+        <is>
+          <t>377.20</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="inlineStr"/>
+      <c r="K80" s="7" t="inlineStr"/>
+      <c r="L80" s="8" t="inlineStr"/>
+      <c r="M80" s="8" t="inlineStr"/>
+      <c r="N80" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O80" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/1f02d0b0-f0c6-4a78-b6da-9b3e50d3cea3.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="55" customHeight="1">
+      <c r="A81" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:35:49.08</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Ambuja Cements Ltd</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr"/>
+      <c r="E81" s="4" t="inlineStr"/>
+      <c r="F81" s="4" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr"/>
+      <c r="H81" s="4" t="inlineStr"/>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>444.25</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr"/>
+      <c r="K81" s="4" t="inlineStr"/>
+      <c r="L81" s="5" t="inlineStr"/>
+      <c r="M81" s="5" t="inlineStr"/>
+      <c r="N81" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O81" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/a9dd70d8-5b6b-420a-8f30-6af84c8909e2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="55" customHeight="1">
+      <c r="A82" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:30:04.637</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>L&amp;T Technology Services Ltd</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr"/>
+      <c r="E82" s="7" t="inlineStr"/>
+      <c r="F82" s="7" t="inlineStr"/>
+      <c r="G82" s="7" t="inlineStr"/>
+      <c r="H82" s="7" t="inlineStr"/>
+      <c r="I82" s="7" t="inlineStr">
+        <is>
+          <t>3802.45</t>
+        </is>
+      </c>
+      <c r="J82" s="7" t="inlineStr"/>
+      <c r="K82" s="7" t="inlineStr"/>
+      <c r="L82" s="8" t="inlineStr"/>
+      <c r="M82" s="8" t="inlineStr"/>
+      <c r="N82" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O82" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/f7fbb8f1-ee4b-4b04-b736-1ea355c99019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="55" customHeight="1">
+      <c r="A83" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:19:56.423</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>ACC Ltd</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr"/>
+      <c r="E83" s="4" t="inlineStr"/>
+      <c r="F83" s="4" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr"/>
+      <c r="H83" s="4" t="inlineStr"/>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>1392.00</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr"/>
+      <c r="K83" s="4" t="inlineStr"/>
+      <c r="L83" s="5" t="inlineStr"/>
+      <c r="M83" s="5" t="inlineStr"/>
+      <c r="N83" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O83" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/a5370bfd-7b6d-4027-89a7-94282b86e47b.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="55" customHeight="1">
+      <c r="A84" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:08:25.22</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>Dhampur Bio Organics Ltd</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr"/>
+      <c r="E84" s="7" t="inlineStr"/>
+      <c r="F84" s="7" t="inlineStr"/>
+      <c r="G84" s="7" t="inlineStr"/>
+      <c r="H84" s="7" t="inlineStr"/>
+      <c r="I84" s="7" t="inlineStr">
+        <is>
+          <t>117.70</t>
+        </is>
+      </c>
+      <c r="J84" s="7" t="inlineStr"/>
+      <c r="K84" s="7" t="inlineStr"/>
+      <c r="L84" s="8" t="inlineStr"/>
+      <c r="M84" s="8" t="inlineStr"/>
+      <c r="N84" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O84" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/da1bb00c-116c-4a80-9e88-66f6356418c8.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="55" customHeight="1">
+      <c r="A85" s="4" t="n">
+        <v>83</v>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:05:20.187</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Sambhv Steel Tubes Ltd</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr"/>
+      <c r="E85" s="4" t="inlineStr"/>
+      <c r="F85" s="4" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr"/>
+      <c r="H85" s="4" t="inlineStr"/>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>129.60</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr"/>
+      <c r="K85" s="4" t="inlineStr"/>
+      <c r="L85" s="5" t="inlineStr"/>
+      <c r="M85" s="5" t="inlineStr"/>
+      <c r="N85" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O85" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/4c3ea38c-757a-46de-9ec5-df7532d96595.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="55" customHeight="1">
+      <c r="A86" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T14:35:58.583</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>Nelcast Ltd</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr"/>
+      <c r="E86" s="7" t="inlineStr"/>
+      <c r="F86" s="7" t="inlineStr"/>
+      <c r="G86" s="7" t="inlineStr"/>
+      <c r="H86" s="7" t="inlineStr"/>
+      <c r="I86" s="7" t="inlineStr">
+        <is>
+          <t>160.00</t>
+        </is>
+      </c>
+      <c r="J86" s="7" t="inlineStr"/>
+      <c r="K86" s="7" t="inlineStr"/>
+      <c r="L86" s="8" t="inlineStr"/>
+      <c r="M86" s="8" t="inlineStr"/>
+      <c r="N86" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O86" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/cf8fcfed-f3b3-4fb9-ba8d-28fa428e64e6.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="55" customHeight="1">
+      <c r="A87" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T14:29:15.743</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Muthoot Capital Services Ltd</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr"/>
+      <c r="E87" s="4" t="inlineStr"/>
+      <c r="F87" s="4" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr"/>
+      <c r="H87" s="4" t="inlineStr"/>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>225.50</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr"/>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="5" t="inlineStr"/>
+      <c r="M87" s="5" t="inlineStr"/>
+      <c r="N87" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O87" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/728e8509-6f4d-4791-a98d-f407935f08ef.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="55" customHeight="1">
+      <c r="A88" s="7" t="n">
+        <v>86</v>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T13:36:22.45</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Mac Charles India Ltd</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr"/>
+      <c r="E88" s="7" t="inlineStr"/>
+      <c r="F88" s="7" t="inlineStr"/>
+      <c r="G88" s="7" t="inlineStr"/>
+      <c r="H88" s="7" t="inlineStr"/>
+      <c r="I88" s="7" t="inlineStr">
+        <is>
+          <t>687.30</t>
+        </is>
+      </c>
+      <c r="J88" s="7" t="inlineStr"/>
+      <c r="K88" s="7" t="inlineStr"/>
+      <c r="L88" s="8" t="inlineStr"/>
+      <c r="M88" s="8" t="inlineStr"/>
+      <c r="N88" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O88" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/c8f33331-de58-4c86-9bbb-837aca64bb0c.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="55" customHeight="1">
+      <c r="A89" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T13:13:24.02</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Bajaj Healthcare Ltd</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr"/>
+      <c r="E89" s="4" t="inlineStr"/>
+      <c r="F89" s="4" t="inlineStr"/>
+      <c r="G89" s="4" t="inlineStr"/>
+      <c r="H89" s="4" t="inlineStr"/>
+      <c r="I89" s="4" t="inlineStr">
+        <is>
+          <t>336.90</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="inlineStr"/>
+      <c r="K89" s="4" t="inlineStr"/>
+      <c r="L89" s="5" t="inlineStr"/>
+      <c r="M89" s="5" t="inlineStr"/>
+      <c r="N89" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O89" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/b4ac9372-7223-4236-9740-2d0b1aeffc8f.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="55" customHeight="1">
+      <c r="A90" s="7" t="n">
+        <v>88</v>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:55:19.213</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>Nukleus Office Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr"/>
+      <c r="E90" s="7" t="inlineStr"/>
+      <c r="F90" s="7" t="inlineStr"/>
+      <c r="G90" s="7" t="inlineStr"/>
+      <c r="H90" s="7" t="inlineStr"/>
+      <c r="I90" s="7" t="inlineStr">
+        <is>
+          <t>211.00</t>
+        </is>
+      </c>
+      <c r="J90" s="7" t="inlineStr"/>
+      <c r="K90" s="7" t="inlineStr"/>
+      <c r="L90" s="8" t="inlineStr"/>
+      <c r="M90" s="8" t="inlineStr"/>
+      <c r="N90" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O90" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/b2f6b6c3-c540-4c00-aae2-39eec5bc5a51.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="55" customHeight="1">
+      <c r="A91" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:54:26.14</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Federal Bank Ltd</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr"/>
+      <c r="E91" s="4" t="inlineStr"/>
+      <c r="F91" s="4" t="inlineStr"/>
+      <c r="G91" s="4" t="inlineStr"/>
+      <c r="H91" s="4" t="inlineStr"/>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>297.30</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="inlineStr"/>
+      <c r="K91" s="4" t="inlineStr"/>
+      <c r="L91" s="5" t="inlineStr"/>
+      <c r="M91" s="5" t="inlineStr"/>
+      <c r="N91" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O91" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/a63f39b7-ca14-440c-8909-9ba8c3a3903a.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="55" customHeight="1">
+      <c r="A92" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:50:43.713</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Ltd</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr"/>
+      <c r="E92" s="7" t="inlineStr"/>
+      <c r="F92" s="7" t="inlineStr"/>
+      <c r="G92" s="7" t="inlineStr"/>
+      <c r="H92" s="7" t="inlineStr"/>
+      <c r="I92" s="7" t="inlineStr">
+        <is>
+          <t>49.46</t>
+        </is>
+      </c>
+      <c r="J92" s="7" t="inlineStr"/>
+      <c r="K92" s="7" t="inlineStr"/>
+      <c r="L92" s="8" t="inlineStr"/>
+      <c r="M92" s="8" t="inlineStr"/>
+      <c r="N92" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O92" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/e1ef9566-fb05-4ec2-a07f-e31c8e12c066.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="55" customHeight="1">
+      <c r="A93" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:49:08.08</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>IFGL Refractories Ltd</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr"/>
+      <c r="E93" s="4" t="inlineStr"/>
+      <c r="F93" s="4" t="inlineStr"/>
+      <c r="G93" s="4" t="inlineStr"/>
+      <c r="H93" s="4" t="inlineStr"/>
+      <c r="I93" s="4" t="inlineStr">
+        <is>
+          <t>191.50</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="inlineStr"/>
+      <c r="K93" s="4" t="inlineStr"/>
+      <c r="L93" s="5" t="inlineStr"/>
+      <c r="M93" s="5" t="inlineStr"/>
+      <c r="N93" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O93" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/699bea45-f8e5-44fa-a9e9-b68eac6949fb.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="55" customHeight="1">
+      <c r="A94" s="7" t="n">
+        <v>92</v>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:48:02.53</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>Nukleus Office Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr"/>
+      <c r="E94" s="7" t="inlineStr"/>
+      <c r="F94" s="7" t="inlineStr"/>
+      <c r="G94" s="7" t="inlineStr"/>
+      <c r="H94" s="7" t="inlineStr"/>
+      <c r="I94" s="7" t="inlineStr">
+        <is>
+          <t>211.00</t>
+        </is>
+      </c>
+      <c r="J94" s="7" t="inlineStr"/>
+      <c r="K94" s="7" t="inlineStr"/>
+      <c r="L94" s="8" t="inlineStr"/>
+      <c r="M94" s="8" t="inlineStr"/>
+      <c r="N94" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O94" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/37f6dc92-69c2-422a-960b-7e91065bd3da.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="55" customHeight="1">
+      <c r="A95" s="4" t="n">
+        <v>93</v>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:44:58.17</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>IFGL Refractories Ltd</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr"/>
+      <c r="E95" s="4" t="inlineStr"/>
+      <c r="F95" s="4" t="inlineStr"/>
+      <c r="G95" s="4" t="inlineStr"/>
+      <c r="H95" s="4" t="inlineStr"/>
+      <c r="I95" s="4" t="inlineStr">
+        <is>
+          <t>191.50</t>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr"/>
+      <c r="K95" s="4" t="inlineStr"/>
+      <c r="L95" s="5" t="inlineStr"/>
+      <c r="M95" s="5" t="inlineStr"/>
+      <c r="N95" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O95" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/e0c00a3d-db38-425c-8ae9-932465ad4057.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="55" customHeight="1">
+      <c r="A96" s="7" t="n">
+        <v>94</v>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:37:39.723</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>Pyramid Technoplast Ltd</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr"/>
+      <c r="E96" s="7" t="inlineStr"/>
+      <c r="F96" s="7" t="inlineStr"/>
+      <c r="G96" s="7" t="inlineStr"/>
+      <c r="H96" s="7" t="inlineStr"/>
+      <c r="I96" s="7" t="inlineStr">
+        <is>
+          <t>176.80</t>
+        </is>
+      </c>
+      <c r="J96" s="7" t="inlineStr"/>
+      <c r="K96" s="7" t="inlineStr"/>
+      <c r="L96" s="8" t="inlineStr"/>
+      <c r="M96" s="8" t="inlineStr"/>
+      <c r="N96" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O96" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/4cf3deb8-e82c-43fc-b1de-c2d78e7d3daa.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="55" customHeight="1">
+      <c r="A97" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:24:43.823</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Modi Naturals Ltd</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr"/>
+      <c r="E97" s="4" t="inlineStr"/>
+      <c r="F97" s="4" t="inlineStr"/>
+      <c r="G97" s="4" t="inlineStr"/>
+      <c r="H97" s="4" t="inlineStr"/>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>376.15</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr"/>
+      <c r="K97" s="4" t="inlineStr"/>
+      <c r="L97" s="5" t="inlineStr"/>
+      <c r="M97" s="5" t="inlineStr"/>
+      <c r="N97" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O97" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/f5dc4ada-c1ce-4d8c-a48b-8acf7e51bb8c.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="55" customHeight="1">
+      <c r="A98" s="7" t="n">
+        <v>96</v>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:16:31.957</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Ltd</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr"/>
+      <c r="E98" s="7" t="inlineStr"/>
+      <c r="F98" s="7" t="inlineStr"/>
+      <c r="G98" s="7" t="inlineStr"/>
+      <c r="H98" s="7" t="inlineStr"/>
+      <c r="I98" s="7" t="inlineStr">
+        <is>
+          <t>49.46</t>
+        </is>
+      </c>
+      <c r="J98" s="7" t="inlineStr"/>
+      <c r="K98" s="7" t="inlineStr"/>
+      <c r="L98" s="8" t="inlineStr"/>
+      <c r="M98" s="8" t="inlineStr"/>
+      <c r="N98" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O98" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/1900624a-454f-4669-8376-88e1d18454dd.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="55" customHeight="1">
+      <c r="A99" s="4" t="n">
+        <v>97</v>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:14:24.997</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Ltd</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr"/>
+      <c r="E99" s="4" t="inlineStr"/>
+      <c r="F99" s="4" t="inlineStr"/>
+      <c r="G99" s="4" t="inlineStr"/>
+      <c r="H99" s="4" t="inlineStr"/>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>49.46</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr"/>
+      <c r="K99" s="4" t="inlineStr"/>
+      <c r="L99" s="5" t="inlineStr"/>
+      <c r="M99" s="5" t="inlineStr"/>
+      <c r="N99" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O99" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/9d00d436-0bd8-43d5-b6c7-5f3f366b13f3.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="55" customHeight="1">
+      <c r="A100" s="7" t="n">
+        <v>98</v>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:11:55.907</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Ltd</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr"/>
+      <c r="E100" s="7" t="inlineStr"/>
+      <c r="F100" s="7" t="inlineStr"/>
+      <c r="G100" s="7" t="inlineStr"/>
+      <c r="H100" s="7" t="inlineStr"/>
+      <c r="I100" s="7" t="inlineStr">
+        <is>
+          <t>49.46</t>
+        </is>
+      </c>
+      <c r="J100" s="7" t="inlineStr"/>
+      <c r="K100" s="7" t="inlineStr"/>
+      <c r="L100" s="8" t="inlineStr"/>
+      <c r="M100" s="8" t="inlineStr"/>
+      <c r="N100" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O100" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/86151cc1-336c-4982-9e41-966f48eb5b74.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="55" customHeight="1">
+      <c r="A101" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:10:03.6</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Ltd</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr"/>
+      <c r="E101" s="4" t="inlineStr"/>
+      <c r="F101" s="4" t="inlineStr"/>
+      <c r="G101" s="4" t="inlineStr"/>
+      <c r="H101" s="4" t="inlineStr"/>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
+          <t>49.46</t>
+        </is>
+      </c>
+      <c r="J101" s="4" t="inlineStr"/>
+      <c r="K101" s="4" t="inlineStr"/>
+      <c r="L101" s="5" t="inlineStr"/>
+      <c r="M101" s="5" t="inlineStr"/>
+      <c r="N101" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O101" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/f3a30cd5-5da1-40c8-85bd-37e7c2ffe7fa.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="55" customHeight="1">
+      <c r="A102" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="B102" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:09:44.93</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>IIFL Capital Services Ltd</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="inlineStr"/>
+      <c r="E102" s="7" t="inlineStr"/>
+      <c r="F102" s="7" t="inlineStr"/>
+      <c r="G102" s="7" t="inlineStr"/>
+      <c r="H102" s="7" t="inlineStr"/>
+      <c r="I102" s="7" t="inlineStr">
+        <is>
+          <t>356.50</t>
+        </is>
+      </c>
+      <c r="J102" s="7" t="inlineStr"/>
+      <c r="K102" s="7" t="inlineStr"/>
+      <c r="L102" s="8" t="inlineStr"/>
+      <c r="M102" s="8" t="inlineStr"/>
+      <c r="N102" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O102" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/af66aba8-05e8-4eb8-9f53-3f9727277d80.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="55" customHeight="1">
+      <c r="A103" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:03:58.943</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Ltd</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr"/>
+      <c r="E103" s="4" t="inlineStr"/>
+      <c r="F103" s="4" t="inlineStr"/>
+      <c r="G103" s="4" t="inlineStr"/>
+      <c r="H103" s="4" t="inlineStr"/>
+      <c r="I103" s="4" t="inlineStr">
+        <is>
+          <t>49.46</t>
+        </is>
+      </c>
+      <c r="J103" s="4" t="inlineStr"/>
+      <c r="K103" s="4" t="inlineStr"/>
+      <c r="L103" s="5" t="inlineStr"/>
+      <c r="M103" s="5" t="inlineStr"/>
+      <c r="N103" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O103" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/bac402f5-318d-4694-9f5c-08cbb1a03e9b.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="55" customHeight="1">
+      <c r="A104" s="7" t="n">
+        <v>102</v>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T11:59:12.83</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>CMS Info Systems Ltd</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="inlineStr"/>
+      <c r="E104" s="7" t="inlineStr"/>
+      <c r="F104" s="7" t="inlineStr"/>
+      <c r="G104" s="7" t="inlineStr"/>
+      <c r="H104" s="7" t="inlineStr"/>
+      <c r="I104" s="7" t="inlineStr">
+        <is>
+          <t>290.00</t>
+        </is>
+      </c>
+      <c r="J104" s="7" t="inlineStr"/>
+      <c r="K104" s="7" t="inlineStr"/>
+      <c r="L104" s="8" t="inlineStr"/>
+      <c r="M104" s="8" t="inlineStr"/>
+      <c r="N104" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O104" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/3783798b-cb9e-444a-8988-1148e91390cf.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="55" customHeight="1">
+      <c r="A105" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T11:53:22.887</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Hindustan Copper Ltd</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr"/>
+      <c r="E105" s="4" t="inlineStr"/>
+      <c r="F105" s="4" t="inlineStr"/>
+      <c r="G105" s="4" t="inlineStr"/>
+      <c r="H105" s="4" t="inlineStr"/>
+      <c r="I105" s="4" t="inlineStr">
+        <is>
+          <t>569.05</t>
+        </is>
+      </c>
+      <c r="J105" s="4" t="inlineStr"/>
+      <c r="K105" s="4" t="inlineStr"/>
+      <c r="L105" s="5" t="inlineStr"/>
+      <c r="M105" s="5" t="inlineStr"/>
+      <c r="N105" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O105" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/69e620c7-326e-4811-a95b-90e4497c2a29.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="55" customHeight="1">
+      <c r="A106" s="7" t="n">
+        <v>104</v>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T11:51:04.577</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>LIC Housing Finance Ltd</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="inlineStr"/>
+      <c r="E106" s="7" t="inlineStr"/>
+      <c r="F106" s="7" t="inlineStr"/>
+      <c r="G106" s="7" t="inlineStr"/>
+      <c r="H106" s="7" t="inlineStr"/>
+      <c r="I106" s="7" t="inlineStr">
+        <is>
+          <t>581.30</t>
+        </is>
+      </c>
+      <c r="J106" s="7" t="inlineStr"/>
+      <c r="K106" s="7" t="inlineStr"/>
+      <c r="L106" s="8" t="inlineStr"/>
+      <c r="M106" s="8" t="inlineStr"/>
+      <c r="N106" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O106" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/46c37883-7f04-4d8b-b386-949663263fc9.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="55" customHeight="1">
+      <c r="A107" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T11:38:21.34</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Vascon Engineers Ltd</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr"/>
+      <c r="E107" s="4" t="inlineStr"/>
+      <c r="F107" s="4" t="inlineStr"/>
+      <c r="G107" s="4" t="inlineStr"/>
+      <c r="H107" s="4" t="inlineStr"/>
+      <c r="I107" s="4" t="inlineStr">
+        <is>
+          <t>39.94</t>
+        </is>
+      </c>
+      <c r="J107" s="4" t="inlineStr"/>
+      <c r="K107" s="4" t="inlineStr"/>
+      <c r="L107" s="5" t="inlineStr"/>
+      <c r="M107" s="5" t="inlineStr"/>
+      <c r="N107" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O107" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/4fc9fecc-4837-4955-a615-51f5d213b63f.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="55" customHeight="1">
+      <c r="A108" s="7" t="n">
+        <v>106</v>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T11:16:03.83</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>IFCI Ltd</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="inlineStr"/>
+      <c r="E108" s="7" t="inlineStr"/>
+      <c r="F108" s="7" t="inlineStr"/>
+      <c r="G108" s="7" t="inlineStr"/>
+      <c r="H108" s="7" t="inlineStr"/>
+      <c r="I108" s="7" t="inlineStr">
+        <is>
+          <t>64.44</t>
+        </is>
+      </c>
+      <c r="J108" s="7" t="inlineStr"/>
+      <c r="K108" s="7" t="inlineStr"/>
+      <c r="L108" s="8" t="inlineStr"/>
+      <c r="M108" s="8" t="inlineStr"/>
+      <c r="N108" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O108" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/6232a51c-63ad-41f3-80a8-6fe4e4d8b855.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="55" customHeight="1">
+      <c r="A109" s="4" t="n">
+        <v>107</v>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T11:11:24.69</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Home First Finance Company India Ltd</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr"/>
+      <c r="E109" s="4" t="inlineStr"/>
+      <c r="F109" s="4" t="inlineStr"/>
+      <c r="G109" s="4" t="inlineStr"/>
+      <c r="H109" s="4" t="inlineStr"/>
+      <c r="I109" s="4" t="inlineStr">
+        <is>
+          <t>1200.00</t>
+        </is>
+      </c>
+      <c r="J109" s="4" t="inlineStr"/>
+      <c r="K109" s="4" t="inlineStr"/>
+      <c r="L109" s="5" t="inlineStr"/>
+      <c r="M109" s="5" t="inlineStr"/>
+      <c r="N109" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O109" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/69567c89-3db1-421b-acc0-16c21cf93ed7.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="55" customHeight="1">
+      <c r="A110" s="7" t="n">
+        <v>108</v>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-10T10:19:58.443</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>Artemis Medicare Services Ltd</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="inlineStr"/>
+      <c r="E110" s="7" t="inlineStr"/>
+      <c r="F110" s="7" t="inlineStr"/>
+      <c r="G110" s="7" t="inlineStr"/>
+      <c r="H110" s="7" t="inlineStr"/>
+      <c r="I110" s="7" t="inlineStr">
+        <is>
+          <t>265.35</t>
+        </is>
+      </c>
+      <c r="J110" s="7" t="inlineStr"/>
+      <c r="K110" s="7" t="inlineStr"/>
+      <c r="L110" s="8" t="inlineStr"/>
+      <c r="M110" s="8" t="inlineStr"/>
+      <c r="N110" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="O110" s="8" t="inlineStr">
         <is>
           <t>https://www.bseindia.com/xml-data/corpfiling/AttachHis/6596af38-642d-43a0-b273-2876b6d932e2.pdf</t>
         </is>

</xml_diff>